<commit_message>
Add movie theming columns and a Florence watch-list tab to Orlando rides sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R1QRKBpTRa9pLKfoTqMHDe
</commit_message>
<xml_diff>
--- a/florida/orlando_theme_park_rides.xlsx
+++ b/florida/orlando_theme_park_rides.xlsx
@@ -9,11 +9,12 @@
   </bookViews>
   <sheets>
     <sheet name="Rides" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Ranked non-rides" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Sources &amp; Notes" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Florence watch list" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Ranked non-rides" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Sources &amp; Notes" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Rides!$A$4:$N$32</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Rides!$A$4:$P$32</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -47,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="319">
   <si>
     <t xml:space="preserve">Orlando theme park rides: EPCOT, Animal Kingdom, Epic Universe (researched Oct 2026)</t>
   </si>
@@ -79,6 +80,12 @@
     <t xml:space="preserve">Florence can ride?</t>
   </si>
   <si>
+    <t xml:space="preserve">Movie / franchise theming</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Watch-ahead pick (rating, notes)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Line-skip system (Disney Lightning Lane / Universal Express)</t>
   </si>
   <si>
@@ -112,6 +119,12 @@
     <t xml:space="preserve">Indoor spinning coaster (reverse launch)</t>
   </si>
   <si>
+    <t xml:space="preserve">Guardians of the Galaxy (Marvel)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guardians of the Galaxy (2014), PG-13. Grown-ups only; Florence can't ride.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lightning Lane Single Pass only (separate purchase)</t>
   </si>
   <si>
@@ -136,6 +149,12 @@
     <t xml:space="preserve">Car-themed high-speed dark ride</t>
   </si>
   <si>
+    <t xml:space="preserve">None (original car-design concept, Chevrolet)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
     <t xml:space="preserve">Multi Pass – Tier 1</t>
   </si>
   <si>
@@ -163,6 +182,9 @@
     <t xml:space="preserve">Hang-glider flight simulator (film)</t>
   </si>
   <si>
+    <t xml:space="preserve">None (aerial film of U.S. landscapes)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Multi Pass – Tier 2</t>
   </si>
   <si>
@@ -187,6 +209,9 @@
     <t xml:space="preserve">No minimum</t>
   </si>
   <si>
+    <t xml:space="preserve">None (original history-of-communication story)</t>
+  </si>
+  <si>
     <t xml:space="preserve">#5 of 20</t>
   </si>
   <si>
@@ -199,6 +224,9 @@
     <t xml:space="preserve">Gentle boat ride through greenhouses</t>
   </si>
   <si>
+    <t xml:space="preserve">None (real greenhouses and farms)</t>
+  </si>
+  <si>
     <t xml:space="preserve">#6 of 20</t>
   </si>
   <si>
@@ -211,6 +239,12 @@
     <t xml:space="preserve">Boat dark ride (small drops)</t>
   </si>
   <si>
+    <t xml:space="preserve">Frozen (2013)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frozen (2013), PG. The ride is set after the film; the short Frozen Fever (2015) fits too. Mildly scary bits: wolves and Marshmallow the snow monster, who also appears on the ride.</t>
+  </si>
+  <si>
     <t xml:space="preserve">No Frozen ride in California</t>
   </si>
   <si>
@@ -229,6 +263,12 @@
     <t xml:space="preserve">Trackless 3D dark ride</t>
   </si>
   <si>
+    <t xml:space="preserve">Ratatouille (2007, Pixar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ratatouille (2007), G. On the ride you're rat-sized and get chased around Gusteau's kitchen: mostly silly, but loud and dark in spots.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Otherwise only at Disneyland Paris</t>
   </si>
   <si>
@@ -247,6 +287,12 @@
     <t xml:space="preserve">Gentle indoor boat ride</t>
   </si>
   <si>
+    <t xml:space="preserve">The Three Caballeros (1944)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Three Caballeros (1944 Disney film, on Disney+). Stars Donald Duck, José Carioca and Panchito; any Donald Duck cartoon is enough prep.</t>
+  </si>
+  <si>
     <t xml:space="preserve">None</t>
   </si>
   <si>
@@ -262,6 +308,9 @@
     <t xml:space="preserve">40" for Green (milder); 44" for Orange (intense centrifuge)</t>
   </si>
   <si>
+    <t xml:space="preserve">None (original Mars mission)</t>
+  </si>
+  <si>
     <t xml:space="preserve">#13 of 20</t>
   </si>
   <si>
@@ -271,6 +320,9 @@
     <t xml:space="preserve">Slow dark ride</t>
   </si>
   <si>
+    <t xml:space="preserve">None (Figment is an original EPCOT character)</t>
+  </si>
+  <si>
     <t xml:space="preserve">#17 of 20</t>
   </si>
   <si>
@@ -280,6 +332,12 @@
     <t xml:space="preserve">Slow clamshell omnimover dark ride + aquarium</t>
   </si>
   <si>
+    <t xml:space="preserve">Finding Nemo (2003, Pixar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finding Nemo (2003), G. The shark and anglerfish scenes are a bit scary for little ones.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Disneyland's Finding Nemo Submarine Voyage is a different ride</t>
   </si>
   <si>
@@ -298,6 +356,12 @@
     <t xml:space="preserve">Open-truck safari through animal savanna</t>
   </si>
   <si>
+    <t xml:space="preserve">None (real live animals)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No movie needed. An African-animals picture book or nature show is a nice primer.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Multi Pass (Animal Kingdom has no tiers)</t>
   </si>
   <si>
@@ -313,6 +377,12 @@
     <t xml:space="preserve">3D flying simulator (motorcycle-style seat)</t>
   </si>
   <si>
+    <t xml:space="preserve">Avatar (2009)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avatar (2009), PG-13. Grown-ups only.</t>
+  </si>
+  <si>
     <t xml:space="preserve">#2 of 8</t>
   </si>
   <si>
@@ -325,6 +395,9 @@
     <t xml:space="preserve">Coaster (forwards and backwards)</t>
   </si>
   <si>
+    <t xml:space="preserve">None (original yeti legend)</t>
+  </si>
+  <si>
     <t xml:space="preserve">No (ended Sept 21, 2026)</t>
   </si>
   <si>
@@ -343,6 +416,9 @@
     <t xml:space="preserve">Slow indoor boat ride</t>
   </si>
   <si>
+    <t xml:space="preserve">Skip the movie for Florence (PG-13). The ride is a calm, glowing-jungle boat trip that needs no backstory.</t>
+  </si>
+  <si>
     <t xml:space="preserve">#6 of 8</t>
   </si>
   <si>
@@ -367,6 +443,12 @@
     <t xml:space="preserve">Short train ride to Conservation Station / Bluey's Wild World</t>
   </si>
   <si>
+    <t xml:space="preserve">Bluey (TV series), since 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bluey (TV-Y, Disney+). Bluey audio plays on the train, and it takes you to Bluey's Wild World. The easiest watch-ahead on this list.</t>
+  </si>
+  <si>
     <t xml:space="preserve">None (a virtual queue was used for Bluey's Wild World access at launch)</t>
   </si>
   <si>
@@ -388,6 +470,12 @@
     <t xml:space="preserve">Trackless lift-vehicle dark ride</t>
   </si>
   <si>
+    <t xml:space="preserve">Harry Potter (set just after Deathly Hallows); the land is 1920s Paris from Fantastic Beasts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Order of the Phoenix (2007), PG-13: introduces Umbridge and the Ministry of Magic. Grown-ups only.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Universal Express (since Aug 2025)</t>
   </si>
   <si>
@@ -409,6 +497,12 @@
     <t xml:space="preserve">Robot-arm dark ride</t>
   </si>
   <si>
+    <t xml:space="preserve">Universal Classic Monsters (Frankenstein, Dracula, etc.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frankenstein (1931) / Bride of Frankenstein (1935). Grown-ups only.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Universal Express</t>
   </si>
   <si>
@@ -424,6 +518,9 @@
     <t xml:space="preserve">Dual-launch racing coaster</t>
   </si>
   <si>
+    <t xml:space="preserve">None (original)</t>
+  </si>
+  <si>
     <t xml:space="preserve">#3 of 11</t>
   </si>
   <si>
@@ -436,6 +533,12 @@
     <t xml:space="preserve">Family coaster with mine-cart 'jumps'</t>
   </si>
   <si>
+    <t xml:space="preserve">Donkey Kong Country (Nintendo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Super Mario Bros. Movie (2023), PG, which features Donkey Kong. Florence can't ride yet, but can see Donkey Kong's land.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Otherwise only at Universal Studios Japan</t>
   </si>
   <si>
@@ -451,6 +554,12 @@
     <t xml:space="preserve">AR/3D interactive dark ride</t>
   </si>
   <si>
+    <t xml:space="preserve">Mario Kart / Super Mario (Nintendo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Super Mario Bros. Movie (2023), PG: Mario, Bowser, and a Rainbow Road kart race.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Same ride at Universal Studios Hollywood's Super Nintendo World</t>
   </si>
   <si>
@@ -466,6 +575,12 @@
     <t xml:space="preserve">Launched family coaster</t>
   </si>
   <si>
+    <t xml:space="preserve">How to Train Your Dragon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How to Train Your Dragon (2010, animated), PG.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Yes (reported dropped at times)</t>
   </si>
   <si>
@@ -484,6 +599,9 @@
     <t xml:space="preserve">No minimum; under 48" need a supervising companion</t>
   </si>
   <si>
+    <t xml:space="preserve">None (original constellation creatures)</t>
+  </si>
+  <si>
     <t xml:space="preserve">#7 of 11</t>
   </si>
   <si>
@@ -499,6 +617,12 @@
     <t xml:space="preserve">40"–48" need a supervising companion</t>
   </si>
   <si>
+    <t xml:space="preserve">Universal Classic Monsters: The Wolf Man (1941)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Wolf Man (1941). Grown-ups only.</t>
+  </si>
+  <si>
     <t xml:space="preserve">#8 of 11</t>
   </si>
   <si>
@@ -511,6 +635,12 @@
     <t xml:space="preserve">Under 48" need a supervising companion</t>
   </si>
   <si>
+    <t xml:space="preserve">Super Mario (Nintendo): Yoshi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Super Mario Galaxy Movie (2026), PG: Yoshi's first big movie role (voiced by Donald Glover).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Otherwise only at Universal Studios Japan (not in Hollywood)</t>
   </si>
   <si>
@@ -541,6 +671,12 @@
     <t xml:space="preserve">Interactive water boat ride (you'll get wet)</t>
   </si>
   <si>
+    <t xml:space="preserve">How to Train Your Dragon (the Viking village of Berk)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How to Train Your Dragon (2010, animated), PG: Hiccup, Toothless and Berk. There's also a 2025 live-action remake (PG). Some intense dragon-battle scenes.</t>
+  </si>
+  <si>
     <t xml:space="preserve">#11 of 11</t>
   </si>
   <si>
@@ -548,6 +684,78 @@
   </si>
   <si>
     <t xml:space="preserve">Rides Florence can do now:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pre-trip watch list for Florence (rides she can do at her current height)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roughly easiest/most toddler-friendly first. The 'Can ride?' column looks up the Rides tab, so it follows the height cell.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Watch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rating</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sets up this ride</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bluey (any episodes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TV-Y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Train to Bluey's Wild World, with Bluey audio on board.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finding Nemo (2003)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shark/anglerfish scenes are a little scary.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ratatouille (2007)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The ride's chase scenes are loud/dark in spots.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frozen (2013) + Frozen Fever short (2015)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wolves and Marshmallow the snow monster may scare her.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Three Caballeros (1944) or Donald Duck shorts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not rated (1944)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Short, gentle ride; Donald familiarity is plenty.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Super Mario Galaxy Movie (2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yoshi's big role. The 2023 Super Mario Bros. Movie (PG) covers the rest of Super Nintendo World.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How to Train Your Dragon (2010, animated)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Some intense dragon battles; Toothless and Berk feature heavily in the land.</t>
   </si>
   <si>
     <t xml:space="preserve">Attractions Wandering in Disney ranks that aren't rides (excluded from the Rides tab)</t>
@@ -1462,7 +1670,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N37"/>
+  <dimension ref="A1:P37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15"/>
@@ -1471,13 +1679,15 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="46"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1540,19 +1750,25 @@
       <c r="N4" s="5" t="s">
         <v>16</v>
       </c>
+      <c r="O4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E5" s="8" t="n">
         <v>42</v>
@@ -1563,39 +1779,45 @@
         <v>Not yet</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="I5" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="J5" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="K5" s="6" t="s">
+      <c r="I5" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="L5" s="8" t="n">
+      <c r="J5" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K5" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="L5" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="M5" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N5" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="M5" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="N5" s="6" t="s">
-        <v>26</v>
+      <c r="O5" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="P5" s="6" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E6" s="8" t="n">
         <v>40</v>
@@ -1606,39 +1828,45 @@
         <v>Not yet</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="I6" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="J6" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="K6" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="L6" s="8" t="n">
+        <v>33</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="K6" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="L6" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="M6" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="N6" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="M6" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="N6" s="6" t="s">
-        <v>34</v>
+      <c r="O6" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="P6" s="6" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="E7" s="8" t="n">
         <v>40</v>
@@ -1649,406 +1877,466 @@
         <v>Not yet</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="I7" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="J7" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="K7" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="L7" s="8" t="n">
+        <v>44</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="K7" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="L7" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="M7" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="N7" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="M7" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="N7" s="6" t="s">
-        <v>41</v>
+      <c r="O7" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="P7" s="6" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E8" s="8"/>
       <c r="F8" s="6" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="G8" s="8" t="str">
         <f aca="false">IF(E8="","Yes",IF($C$2&gt;=E8,"Yes","Not yet"))</f>
         <v>Yes</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="I8" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="J8" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K8" s="6"/>
-      <c r="L8" s="8" t="n">
+        <v>53</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="L8" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="M8" s="6"/>
+      <c r="N8" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="M8" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="N8" s="6" t="s">
-        <v>47</v>
+      <c r="O8" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="P8" s="6" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="E9" s="8"/>
       <c r="F9" s="6" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="G9" s="8" t="str">
         <f aca="false">IF(E9="","Yes",IF($C$2&gt;=E9,"Yes","Not yet"))</f>
         <v>Yes</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="I9" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="J9" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K9" s="6"/>
-      <c r="L9" s="8" t="n">
+        <v>58</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="K9" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="L9" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="M9" s="6"/>
+      <c r="N9" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="M9" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="N9" s="6"/>
-    </row>
-    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O9" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="P9" s="6"/>
+    </row>
+    <row r="10" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="E10" s="8"/>
       <c r="F10" s="6" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="G10" s="8" t="str">
         <f aca="false">IF(E10="","Yes",IF($C$2&gt;=E10,"Yes","Not yet"))</f>
         <v>Yes</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="I10" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="J10" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K10" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="L10" s="8" t="n">
+        <v>63</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="K10" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="L10" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="M10" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="N10" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="M10" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="N10" s="6" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O10" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="P10" s="6" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="E11" s="8"/>
       <c r="F11" s="6" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="G11" s="8" t="str">
         <f aca="false">IF(E11="","Yes",IF($C$2&gt;=E11,"Yes","Not yet"))</f>
         <v>Yes</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="I11" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="J11" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K11" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="L11" s="8" t="n">
+        <v>71</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="K11" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="L11" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="M11" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="N11" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="M11" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="N11" s="6" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O11" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="P11" s="6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="E12" s="8"/>
       <c r="F12" s="6" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="G12" s="8" t="str">
         <f aca="false">IF(E12="","Yes",IF($C$2&gt;=E12,"Yes","Not yet"))</f>
         <v>Yes</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="I12" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="J12" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K12" s="6"/>
-      <c r="L12" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="K12" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="L12" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="M12" s="6"/>
+      <c r="N12" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="M12" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="N12" s="6"/>
+      <c r="O12" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="P12" s="6"/>
     </row>
     <row r="13" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="E13" s="8" t="n">
         <v>40</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="G13" s="8" t="str">
         <f aca="false">IF(E13="","Yes",IF($C$2&gt;=E13,"Yes","Not yet"))</f>
         <v>Not yet</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="I13" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="J13" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K13" s="6"/>
-      <c r="L13" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="K13" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="L13" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="M13" s="6"/>
+      <c r="N13" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="M13" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="N13" s="6"/>
+      <c r="O13" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="P13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="E14" s="8"/>
       <c r="F14" s="6" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="G14" s="8" t="str">
         <f aca="false">IF(E14="","Yes",IF($C$2&gt;=E14,"Yes","Not yet"))</f>
         <v>Yes</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="I14" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="J14" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="K14" s="6"/>
-      <c r="L14" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="K14" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="L14" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="M14" s="6"/>
+      <c r="N14" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="M14" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="N14" s="6"/>
+      <c r="O14" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="P14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>76</v>
+        <v>93</v>
       </c>
       <c r="E15" s="8"/>
       <c r="F15" s="6" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="G15" s="8" t="str">
         <f aca="false">IF(E15="","Yes",IF($C$2&gt;=E15,"Yes","Not yet"))</f>
         <v>Yes</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="I15" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="J15" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="K15" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="L15" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="K15" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="L15" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="M15" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="N15" s="8" t="n">
         <v>11</v>
       </c>
-      <c r="M15" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="N15" s="6"/>
+      <c r="O15" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="P15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>81</v>
+        <v>100</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>82</v>
+        <v>101</v>
       </c>
       <c r="E16" s="11"/>
       <c r="F16" s="9" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="G16" s="11" t="str">
         <f aca="false">IF(E16="","Yes",IF($C$2&gt;=E16,"Yes","Not yet"))</f>
         <v>Yes</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="I16" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="J16" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="K16" s="9"/>
-      <c r="L16" s="11" t="n">
+        <v>102</v>
+      </c>
+      <c r="I16" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="J16" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="K16" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="L16" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="M16" s="9"/>
+      <c r="N16" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="M16" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="N16" s="9" t="s">
-        <v>26</v>
+      <c r="O16" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="P16" s="9" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>85</v>
+        <v>106</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>86</v>
+        <v>107</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>87</v>
+        <v>108</v>
       </c>
       <c r="E17" s="11" t="n">
         <v>44</v>
@@ -2059,35 +2347,41 @@
         <v>Not yet</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="I17" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="J17" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="K17" s="9"/>
-      <c r="L17" s="11" t="n">
+        <v>109</v>
+      </c>
+      <c r="I17" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="J17" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="K17" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="L17" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="M17" s="9"/>
+      <c r="N17" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="M17" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="N17" s="9"/>
+      <c r="O17" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="P17" s="9"/>
     </row>
     <row r="18" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>89</v>
+        <v>112</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
       <c r="E18" s="11" t="n">
         <v>44</v>
@@ -2098,78 +2392,90 @@
         <v>Not yet</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="I18" s="11" t="s">
-        <v>92</v>
-      </c>
-      <c r="J18" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="K18" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="L18" s="11" t="n">
+        <v>115</v>
+      </c>
+      <c r="I18" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="J18" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="K18" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="L18" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="M18" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="N18" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="M18" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="N18" s="9" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O18" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="P18" s="9" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>85</v>
+        <v>106</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="E19" s="11"/>
       <c r="F19" s="9" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="G19" s="11" t="str">
         <f aca="false">IF(E19="","Yes",IF($C$2&gt;=E19,"Yes","Not yet"))</f>
         <v>Yes</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="I19" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="J19" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="K19" s="9"/>
-      <c r="L19" s="11" t="n">
+        <v>109</v>
+      </c>
+      <c r="I19" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="J19" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="K19" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="L19" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="M19" s="9"/>
+      <c r="N19" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="M19" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="N19" s="9"/>
+      <c r="O19" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="P19" s="9"/>
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>89</v>
+        <v>112</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>99</v>
+        <v>124</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>100</v>
+        <v>125</v>
       </c>
       <c r="E20" s="11" t="n">
         <v>38</v>
@@ -2180,76 +2486,88 @@
         <v>Not yet</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="I20" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="J20" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="K20" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="L20" s="11" t="n">
+        <v>81</v>
+      </c>
+      <c r="I20" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="J20" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="K20" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="L20" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="M20" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="N20" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="M20" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="N20" s="9"/>
+      <c r="O20" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="P20" s="9"/>
     </row>
     <row r="21" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>103</v>
+        <v>128</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>104</v>
+        <v>129</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>105</v>
+        <v>130</v>
       </c>
       <c r="E21" s="11"/>
       <c r="F21" s="9" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="G21" s="11" t="str">
         <f aca="false">IF(E21="","Yes",IF($C$2&gt;=E21,"Yes","Not yet"))</f>
         <v>Yes</v>
       </c>
       <c r="H21" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="I21" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="J21" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="K21" s="9"/>
-      <c r="L21" s="11"/>
-      <c r="M21" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="N21" s="9" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>131</v>
+      </c>
+      <c r="I21" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="J21" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="K21" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="L21" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="M21" s="9"/>
+      <c r="N21" s="11"/>
+      <c r="O21" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="P21" s="9" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>109</v>
+        <v>136</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>110</v>
+        <v>137</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>111</v>
+        <v>138</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>112</v>
+        <v>139</v>
       </c>
       <c r="E22" s="14" t="n">
         <v>40</v>
@@ -2260,39 +2578,45 @@
         <v>Not yet</v>
       </c>
       <c r="H22" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="I22" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="J22" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="K22" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="L22" s="14" t="n">
+        <v>140</v>
+      </c>
+      <c r="I22" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="J22" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="K22" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="L22" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="M22" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="N22" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="M22" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="N22" s="12" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O22" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="P22" s="12" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>109</v>
+        <v>136</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>117</v>
+        <v>146</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>118</v>
+        <v>147</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>119</v>
+        <v>148</v>
       </c>
       <c r="E23" s="14" t="n">
         <v>48</v>
@@ -2303,35 +2627,41 @@
         <v>Not yet</v>
       </c>
       <c r="H23" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="I23" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="J23" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K23" s="12"/>
-      <c r="L23" s="14" t="n">
+        <v>149</v>
+      </c>
+      <c r="I23" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="J23" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="K23" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="L23" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="M23" s="12"/>
+      <c r="N23" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="M23" s="14" t="s">
-        <v>121</v>
-      </c>
-      <c r="N23" s="12"/>
+      <c r="O23" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="P23" s="12"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
-        <v>109</v>
+        <v>136</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>122</v>
+        <v>153</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>123</v>
+        <v>154</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>124</v>
+        <v>155</v>
       </c>
       <c r="E24" s="14" t="n">
         <v>48</v>
@@ -2342,35 +2672,41 @@
         <v>Not yet</v>
       </c>
       <c r="H24" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="I24" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="J24" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K24" s="12"/>
-      <c r="L24" s="14" t="n">
+        <v>156</v>
+      </c>
+      <c r="I24" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="J24" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="K24" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="L24" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="M24" s="12"/>
+      <c r="N24" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="M24" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="N24" s="12"/>
+      <c r="O24" s="14" t="s">
+        <v>157</v>
+      </c>
+      <c r="P24" s="12"/>
     </row>
     <row r="25" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>109</v>
+        <v>136</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>126</v>
+        <v>158</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>127</v>
+        <v>159</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>128</v>
+        <v>160</v>
       </c>
       <c r="E25" s="14" t="n">
         <v>40</v>
@@ -2381,37 +2717,43 @@
         <v>Not yet</v>
       </c>
       <c r="H25" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="I25" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="J25" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K25" s="12" t="s">
-        <v>129</v>
-      </c>
-      <c r="L25" s="14" t="n">
+        <v>161</v>
+      </c>
+      <c r="I25" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="J25" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="K25" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="L25" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="M25" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="N25" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="M25" s="14" t="s">
-        <v>130</v>
-      </c>
-      <c r="N25" s="12"/>
+      <c r="O25" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="P25" s="12"/>
     </row>
     <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>109</v>
+        <v>136</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>131</v>
+        <v>165</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>132</v>
+        <v>166</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>133</v>
+        <v>167</v>
       </c>
       <c r="E26" s="14" t="n">
         <v>40</v>
@@ -2422,37 +2764,43 @@
         <v>Not yet</v>
       </c>
       <c r="H26" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="I26" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="J26" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="K26" s="12" t="s">
-        <v>134</v>
-      </c>
-      <c r="L26" s="14" t="n">
+        <v>168</v>
+      </c>
+      <c r="I26" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="J26" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="K26" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="L26" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="M26" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="N26" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="M26" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="N26" s="12"/>
+      <c r="O26" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="P26" s="12"/>
     </row>
     <row r="27" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>109</v>
+        <v>136</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>136</v>
+        <v>172</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>137</v>
+        <v>173</v>
       </c>
       <c r="D27" s="12" t="s">
-        <v>138</v>
+        <v>174</v>
       </c>
       <c r="E27" s="14" t="n">
         <v>40</v>
@@ -2463,164 +2811,188 @@
         <v>Not yet</v>
       </c>
       <c r="H27" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="I27" s="14" t="s">
-        <v>139</v>
-      </c>
-      <c r="J27" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K27" s="12"/>
-      <c r="L27" s="14" t="n">
+        <v>175</v>
+      </c>
+      <c r="I27" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="J27" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="K27" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="L27" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="M27" s="12"/>
+      <c r="N27" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="M27" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="N27" s="12" t="s">
-        <v>141</v>
+      <c r="O27" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="P27" s="12" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>109</v>
+        <v>136</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>122</v>
+        <v>153</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>142</v>
+        <v>180</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>143</v>
+        <v>181</v>
       </c>
       <c r="E28" s="14"/>
       <c r="F28" s="12" t="s">
-        <v>144</v>
+        <v>182</v>
       </c>
       <c r="G28" s="14" t="str">
         <f aca="false">IF(E28="","Yes",IF($C$2&gt;=E28,"Yes","Not yet"))</f>
         <v>Yes</v>
       </c>
       <c r="H28" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="I28" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="J28" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K28" s="12"/>
-      <c r="L28" s="14" t="n">
+        <v>183</v>
+      </c>
+      <c r="I28" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="J28" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="K28" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="L28" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="M28" s="12"/>
+      <c r="N28" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="M28" s="14" t="s">
-        <v>145</v>
-      </c>
-      <c r="N28" s="12" t="s">
+      <c r="O28" s="14" t="s">
+        <v>184</v>
+      </c>
+      <c r="P28" s="12" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="B29" s="12" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="B29" s="12" t="s">
-        <v>117</v>
-      </c>
       <c r="C29" s="13" t="s">
-        <v>147</v>
+        <v>186</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>148</v>
+        <v>187</v>
       </c>
       <c r="E29" s="14" t="n">
         <v>40</v>
       </c>
       <c r="F29" s="12" t="s">
-        <v>149</v>
+        <v>188</v>
       </c>
       <c r="G29" s="14" t="str">
         <f aca="false">IF(E29="","Yes",IF($C$2&gt;=E29,"Yes","Not yet"))</f>
         <v>Not yet</v>
       </c>
       <c r="H29" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="I29" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="J29" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K29" s="12"/>
-      <c r="L29" s="14" t="n">
+        <v>189</v>
+      </c>
+      <c r="I29" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="J29" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="K29" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="L29" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="M29" s="12"/>
+      <c r="N29" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="M29" s="14" t="s">
-        <v>150</v>
-      </c>
-      <c r="N29" s="12"/>
-    </row>
-    <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O29" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="P29" s="12"/>
+    </row>
+    <row r="30" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>109</v>
+        <v>136</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>131</v>
+        <v>165</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>151</v>
+        <v>192</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>152</v>
+        <v>193</v>
       </c>
       <c r="E30" s="14" t="n">
         <v>34</v>
       </c>
       <c r="F30" s="12" t="s">
-        <v>153</v>
+        <v>194</v>
       </c>
       <c r="G30" s="14" t="str">
         <f aca="false">IF(E30="","Yes",IF($C$2&gt;=E30,"Yes","Not yet"))</f>
         <v>Yes</v>
       </c>
       <c r="H30" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="I30" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="J30" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K30" s="12" t="s">
-        <v>154</v>
-      </c>
-      <c r="L30" s="14" t="n">
+        <v>195</v>
+      </c>
+      <c r="I30" s="12" t="s">
+        <v>196</v>
+      </c>
+      <c r="J30" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="K30" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="L30" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="M30" s="12" t="s">
+        <v>197</v>
+      </c>
+      <c r="N30" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="M30" s="14" t="s">
-        <v>155</v>
-      </c>
-      <c r="N30" s="12" t="s">
-        <v>156</v>
+      <c r="O30" s="14" t="s">
+        <v>198</v>
+      </c>
+      <c r="P30" s="12" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
-        <v>109</v>
+        <v>136</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>136</v>
+        <v>172</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>157</v>
+        <v>200</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>158</v>
+        <v>201</v>
       </c>
       <c r="E31" s="14" t="n">
         <v>48</v>
@@ -2631,74 +3003,86 @@
         <v>Not yet</v>
       </c>
       <c r="H31" s="12" t="s">
-        <v>159</v>
-      </c>
-      <c r="I31" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="J31" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K31" s="12"/>
-      <c r="L31" s="14" t="n">
+        <v>175</v>
+      </c>
+      <c r="I31" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="J31" s="12" t="s">
+        <v>202</v>
+      </c>
+      <c r="K31" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="L31" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="M31" s="12"/>
+      <c r="N31" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="M31" s="14" t="s">
-        <v>160</v>
-      </c>
-      <c r="N31" s="12" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O31" s="14" t="s">
+        <v>203</v>
+      </c>
+      <c r="P31" s="12" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>109</v>
+        <v>136</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>136</v>
+        <v>172</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>162</v>
+        <v>205</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>163</v>
+        <v>206</v>
       </c>
       <c r="E32" s="14"/>
       <c r="F32" s="12" t="s">
-        <v>144</v>
+        <v>182</v>
       </c>
       <c r="G32" s="14" t="str">
         <f aca="false">IF(E32="","Yes",IF($C$2&gt;=E32,"Yes","Not yet"))</f>
         <v>Yes</v>
       </c>
       <c r="H32" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="I32" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="J32" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K32" s="12"/>
-      <c r="L32" s="14" t="n">
+        <v>207</v>
+      </c>
+      <c r="I32" s="12" t="s">
+        <v>208</v>
+      </c>
+      <c r="J32" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="K32" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="L32" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="M32" s="12"/>
+      <c r="N32" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="M32" s="14" t="s">
-        <v>164</v>
-      </c>
-      <c r="N32" s="12" t="s">
-        <v>165</v>
+      <c r="O32" s="14" t="s">
+        <v>209</v>
+      </c>
+      <c r="P32" s="12" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="15" t="s">
-        <v>166</v>
+        <v>211</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="16" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B35" s="16" t="str">
         <f aca="false">COUNTIFS($A$5:$A$32,A35,$G$5:$G$32,"Yes")&amp;" of "&amp;COUNTIF($A$5:$A$32,A35)</f>
@@ -2707,7 +3091,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="16" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="B36" s="16" t="str">
         <f aca="false">COUNTIFS($A$5:$A$32,A36,$G$5:$G$32,"Yes")&amp;" of "&amp;COUNTIF($A$5:$A$32,A36)</f>
@@ -2716,7 +3100,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="16" t="s">
-        <v>109</v>
+        <v>136</v>
       </c>
       <c r="B37" s="16" t="str">
         <f aca="false">COUNTIFS($A$5:$A$32,A37,$G$5:$G$32,"Yes")&amp;" of "&amp;COUNTIF($A$5:$A$32,A37)</f>
@@ -2724,7 +3108,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:N32"/>
+  <autoFilter ref="A4:P32"/>
   <mergeCells count="1">
     <mergeCell ref="A2:B2"/>
   </mergeCells>
@@ -2736,9 +3120,9 @@
       <formula>G5="Not yet"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J5:J32">
+  <conditionalFormatting sqref="L5:L32">
     <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
-      <formula>J5="Yes"</formula>
+      <formula>L5="Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2758,213 +3142,203 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="56"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="17" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="18" t="s">
+        <v>214</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>216</v>
+      </c>
+      <c r="D4" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="18" t="s">
-        <v>168</v>
-      </c>
-      <c r="C3" s="18" t="s">
-        <v>169</v>
-      </c>
-      <c r="D3" s="18" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="19" t="s">
-        <v>170</v>
-      </c>
-      <c r="C4" s="19" t="s">
-        <v>171</v>
-      </c>
-      <c r="D4" s="19" t="s">
-        <v>172</v>
+      <c r="E4" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="18" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="19" t="s">
-        <v>173</v>
-      </c>
-      <c r="C5" s="19" t="s">
-        <v>174</v>
-      </c>
-      <c r="D5" s="19" t="s">
-        <v>175</v>
+      <c r="A5" s="10" t="s">
+        <v>218</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="E5" s="11" t="str">
+        <f aca="false">IFERROR(INDEX(Rides!$G$5:$G$32,MATCH(C5,Rides!$C$5:$C$32,0)),"?")</f>
+        <v>Yes</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="19" t="s">
-        <v>176</v>
-      </c>
-      <c r="C6" s="19" t="s">
-        <v>177</v>
-      </c>
-      <c r="D6" s="19" t="s">
-        <v>178</v>
+      <c r="A6" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="8" t="str">
+        <f aca="false">IFERROR(INDEX(Rides!$G$5:$G$32,MATCH(C6,Rides!$C$5:$C$32,0)),"?")</f>
+        <v>Yes</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="19" t="s">
-        <v>179</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>180</v>
-      </c>
-      <c r="D7" s="19" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="19" t="s">
-        <v>182</v>
-      </c>
-      <c r="C8" s="19" t="s">
-        <v>180</v>
-      </c>
-      <c r="D8" s="19" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9" s="19" t="s">
-        <v>184</v>
-      </c>
-      <c r="C9" s="19" t="s">
-        <v>185</v>
-      </c>
-      <c r="D9" s="19" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" s="19" t="s">
-        <v>187</v>
-      </c>
-      <c r="C10" s="19" t="s">
-        <v>188</v>
-      </c>
-      <c r="D10" s="19" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" s="19" t="s">
-        <v>190</v>
-      </c>
-      <c r="C11" s="19" t="s">
-        <v>191</v>
-      </c>
-      <c r="D11" s="19" t="s">
+      <c r="A7" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="8" t="str">
+        <f aca="false">IFERROR(INDEX(Rides!$G$5:$G$32,MATCH(C7,Rides!$C$5:$C$32,0)),"?")</f>
+        <v>Yes</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="8" t="str">
+        <f aca="false">IFERROR(INDEX(Rides!$G$5:$G$32,MATCH(C8,Rides!$C$5:$C$32,0)),"?")</f>
+        <v>Yes</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="8" t="str">
+        <f aca="false">IFERROR(INDEX(Rides!$G$5:$G$32,MATCH(C9,Rides!$C$5:$C$32,0)),"?")</f>
+        <v>Yes</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13" t="s">
+        <v>232</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="C10" s="12" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12" s="19" t="s">
-        <v>193</v>
-      </c>
-      <c r="C12" s="19" t="s">
-        <v>194</v>
-      </c>
-      <c r="D12" s="19" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="20" t="s">
-        <v>79</v>
-      </c>
-      <c r="B13" s="20" t="s">
-        <v>196</v>
-      </c>
-      <c r="C13" s="20" t="s">
-        <v>197</v>
-      </c>
-      <c r="D13" s="20" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20" t="s">
-        <v>79</v>
-      </c>
-      <c r="B14" s="20" t="s">
-        <v>199</v>
-      </c>
-      <c r="C14" s="20" t="s">
-        <v>200</v>
-      </c>
-      <c r="D14" s="20" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="20" t="s">
-        <v>79</v>
-      </c>
-      <c r="B15" s="20" t="s">
-        <v>202</v>
-      </c>
-      <c r="C15" s="20" t="s">
-        <v>203</v>
-      </c>
-      <c r="D15" s="20" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="15" t="s">
+      <c r="D10" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="E10" s="14" t="str">
+        <f aca="false">IFERROR(INDEX(Rides!$G$5:$G$32,MATCH(C10,Rides!$C$5:$C$32,0)),"?")</f>
+        <v>Yes</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="13" t="s">
+        <v>234</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="C11" s="12" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="16" t="s">
-        <v>206</v>
+      <c r="D11" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="E11" s="14" t="str">
+        <f aca="false">IFERROR(INDEX(Rides!$G$5:$G$32,MATCH(C11,Rides!$C$5:$C$32,0)),"?")</f>
+        <v>Yes</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>235</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="E5:E11">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+      <formula>E5="Yes"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
+      <formula>E5="Not yet"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2980,6 +3354,228 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="17" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>237</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>238</v>
+      </c>
+      <c r="D3" s="18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="19" t="s">
+        <v>239</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>240</v>
+      </c>
+      <c r="D4" s="19" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>242</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>243</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>245</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>246</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>248</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>249</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>251</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>249</v>
+      </c>
+      <c r="D8" s="19" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>253</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>254</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="19" t="s">
+        <v>256</v>
+      </c>
+      <c r="C10" s="19" t="s">
+        <v>257</v>
+      </c>
+      <c r="D10" s="19" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" s="19" t="s">
+        <v>259</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>260</v>
+      </c>
+      <c r="D11" s="19" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="19" t="s">
+        <v>262</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>263</v>
+      </c>
+      <c r="D12" s="19" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="B13" s="20" t="s">
+        <v>265</v>
+      </c>
+      <c r="C13" s="20" t="s">
+        <v>266</v>
+      </c>
+      <c r="D13" s="20" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="B14" s="20" t="s">
+        <v>268</v>
+      </c>
+      <c r="C14" s="20" t="s">
+        <v>269</v>
+      </c>
+      <c r="D14" s="20" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="B15" s="20" t="s">
+        <v>271</v>
+      </c>
+      <c r="C15" s="20" t="s">
+        <v>272</v>
+      </c>
+      <c r="D15" s="20" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="15" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="16" t="s">
+        <v>275</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:B26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -2989,7 +3585,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="21" t="s">
-        <v>207</v>
+        <v>276</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2997,7 +3593,7 @@
         <v>7</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>208</v>
+        <v>277</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3005,55 +3601,55 @@
         <v>9</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>209</v>
+        <v>278</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="22" t="s">
-        <v>210</v>
+        <v>279</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>211</v>
+        <v>280</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="22" t="s">
-        <v>212</v>
+        <v>281</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>213</v>
+        <v>282</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="s">
-        <v>214</v>
+        <v>283</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>215</v>
+        <v>284</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22" t="s">
-        <v>216</v>
+        <v>285</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>217</v>
+        <v>286</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="s">
-        <v>218</v>
+        <v>287</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>219</v>
+        <v>288</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="22" t="s">
-        <v>220</v>
+        <v>289</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>221</v>
+        <v>290</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3061,111 +3657,111 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="21" t="s">
-        <v>222</v>
+        <v>291</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="22" t="s">
-        <v>223</v>
+        <v>292</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>224</v>
+        <v>293</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="22" t="s">
-        <v>225</v>
+        <v>294</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>226</v>
+        <v>295</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="22" t="s">
-        <v>227</v>
+        <v>296</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>228</v>
+        <v>297</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="22" t="s">
-        <v>229</v>
+        <v>298</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>230</v>
+        <v>299</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="22" t="s">
-        <v>231</v>
+        <v>300</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>232</v>
+        <v>301</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="22" t="s">
-        <v>233</v>
+        <v>302</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>234</v>
+        <v>303</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="22" t="s">
-        <v>235</v>
+        <v>304</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>236</v>
+        <v>305</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="22" t="s">
-        <v>237</v>
+        <v>306</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>238</v>
+        <v>307</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="22" t="s">
-        <v>239</v>
+        <v>308</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>240</v>
+        <v>309</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="22" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>241</v>
+        <v>310</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="22" t="s">
-        <v>242</v>
+        <v>311</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>243</v>
+        <v>312</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="22" t="s">
-        <v>244</v>
+        <v>313</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>245</v>
+        <v>314</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="22" t="s">
-        <v>246</v>
+        <v>315</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>247</v>
+        <v>316</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3173,10 +3769,10 @@
     </row>
     <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="22" t="s">
-        <v>248</v>
+        <v>317</v>
       </c>
       <c r="B26" s="23" t="s">
-        <v>249</v>
+        <v>318</v>
       </c>
     </row>
   </sheetData>

</xml_diff>